<commit_message>
Fix MathVerse judge parsing in benchmark scorer
</commit_message>
<xml_diff>
--- a/results/qwen25vl3b_7b_answer_grpo_selected25_greedy_temp06.xlsx
+++ b/results/qwen25vl3b_7b_answer_grpo_selected25_greedy_temp06.xlsx
@@ -428,15 +428,6 @@
   </sheetPr>
   <dimension ref="A1:G26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="24" customWidth="1" min="1" max="1"/>
-    <col width="18" customWidth="1" min="2" max="2"/>
-    <col width="24" customWidth="1" min="3" max="3"/>
-    <col width="18" customWidth="1" min="4" max="4"/>
-    <col width="24" customWidth="1" min="5" max="5"/>
-    <col width="12" customWidth="1" min="6" max="6"/>
-    <col width="12" customWidth="1" min="7" max="7"/>
-  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
@@ -1113,15 +1104,6 @@
   </sheetPr>
   <dimension ref="A1:G26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="24" customWidth="1" min="1" max="1"/>
-    <col width="18" customWidth="1" min="2" max="2"/>
-    <col width="24" customWidth="1" min="3" max="3"/>
-    <col width="18" customWidth="1" min="4" max="4"/>
-    <col width="24" customWidth="1" min="5" max="5"/>
-    <col width="12" customWidth="1" min="6" max="6"/>
-    <col width="12" customWidth="1" min="7" max="7"/>
-  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
@@ -1417,22 +1399,22 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>19.0355</v>
+        <v>34.1371</v>
       </c>
       <c r="C12" t="n">
-        <v>21.3198</v>
+        <v>38.0711</v>
       </c>
       <c r="D12" t="n">
-        <v>25.2538</v>
+        <v>43.6548</v>
       </c>
       <c r="E12" t="n">
-        <v>24.7462</v>
+        <v>45.1777</v>
       </c>
       <c r="F12" t="n">
-        <v>2.2843</v>
+        <v>3.934</v>
       </c>
       <c r="G12" t="n">
-        <v>-0.5076000000000001</v>
+        <v>1.5229</v>
       </c>
     </row>
     <row r="13">

</xml_diff>

<commit_message>
Repair deterministic benchmark score parsing
</commit_message>
<xml_diff>
--- a/results/qwen25vl3b_7b_answer_grpo_selected25_greedy_temp06.xlsx
+++ b/results/qwen25vl3b_7b_answer_grpo_selected25_greedy_temp06.xlsx
@@ -1599,22 +1599,22 @@
         </is>
       </c>
       <c r="B20" t="n">
-        <v>50</v>
+        <v>64.9371</v>
       </c>
       <c r="C20" t="n">
-        <v>54.3239</v>
+        <v>64.2296</v>
       </c>
       <c r="D20" t="n">
-        <v>77.12260000000001</v>
+        <v>77.2013</v>
       </c>
       <c r="E20" t="n">
-        <v>77.8302</v>
+        <v>77.673</v>
       </c>
       <c r="F20" t="n">
-        <v>4.3239</v>
+        <v>-0.707499999999996</v>
       </c>
       <c r="G20" t="n">
-        <v>0.7075</v>
+        <v>0.4716999999999985</v>
       </c>
     </row>
     <row r="21">
@@ -1661,10 +1661,10 @@
         <v>78.13330000000001</v>
       </c>
       <c r="F22" t="n">
-        <v>2.8534</v>
+        <v>2.853400000000008</v>
       </c>
       <c r="G22" t="n">
-        <v>4.5067</v>
+        <v>4.506600000000006</v>
       </c>
     </row>
     <row r="23">

</xml_diff>

<commit_message>
Repair VisualPuzzles LLM extraction scoring
</commit_message>
<xml_diff>
--- a/results/qwen25vl3b_7b_answer_grpo_selected25_greedy_temp06.xlsx
+++ b/results/qwen25vl3b_7b_answer_grpo_selected25_greedy_temp06.xlsx
@@ -1699,22 +1699,22 @@
         </is>
       </c>
       <c r="B24" t="n">
-        <v>16.0959</v>
+        <v>17.12328767123288</v>
       </c>
       <c r="C24" t="n">
-        <v>18.5788</v>
+        <v>20.80479452054794</v>
       </c>
       <c r="D24" t="n">
-        <v>18.2363</v>
+        <v>20.03424657534246</v>
       </c>
       <c r="E24" t="n">
-        <v>20.5479</v>
+        <v>22.77397260273973</v>
       </c>
       <c r="F24" t="n">
-        <v>2.4829</v>
+        <v>3.681506849315067</v>
       </c>
       <c r="G24" t="n">
-        <v>2.3116</v>
+        <v>2.739726027397261</v>
       </c>
     </row>
     <row r="25">

</xml_diff>